<commit_message>
Add email notification step to the HVAC lead Make.com scenarios
Fabien: needs an email when leads come in, on top of the sheet row,
since the 15-minute SLA depends on him actually knowing a lead
arrived. Added as a second action in each Make.com scenario (Gmail
Send an Email to fabien@halostrategic.com, right after Add a Row),
documented in the tracker's Make.com Setup tab and the brief. Not
built or tested, no Make.com/Gmail access in this session.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014zdMVC2PGgF2M5N7pSgc3d
</commit_message>
<xml_diff>
--- a/halo-growth-hvac/hvac-qualified-lead-tracker.xlsx
+++ b/halo-growth-hvac/hvac-qualified-lead-tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="73">
   <si>
     <t xml:space="preserve">Halo Strategic — US HVAC LinkedIn Campaign</t>
   </si>
@@ -211,10 +211,10 @@
     <t xml:space="preserve">Connecting LinkedIn Lead Gen Forms to this sheet via Make.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Decided: two separate Lead Gen Forms (one per ad), each with its own Make scenario, so Concept A/C attribution is automatic rather than guessed. I have no LinkedIn or Make.com access in this session, so this hasn't been built or tested; verify against Make's actual current UI as you go.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0. In Campaign Manager, build two Lead Gen Forms with identical content (same fields, headline, supporting copy, confirmation message from CLAUDE_BROWSER_LINKEDIN_BRIEF.md), one attached to Ad 1 (Concept A) and one to Ad 2 (Concept C). This replaces the earlier one-shared-form plan, needed so each Make scenario can watch its own form and know which concept it belongs to.</t>
+    <t xml:space="preserve">Decided: two separate Lead Gen Forms (one per ad), each with its own Make scenario, plus an email notification to Fabien on every new lead. I have no LinkedIn, Make.com, or Gmail access in this session, so this hasn't been built or tested; verify against Make's actual current UI as you go.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0. In Campaign Manager, build two Lead Gen Forms with identical content (same fields, headline, supporting copy, confirmation message from CLAUDE_BROWSER_LINKEDIN_BRIEF.md), one attached to Ad 1 (Concept A) and one to Ad 2 (Concept C). Needed so each Make scenario can watch its own form and know which concept it belongs to.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Import this file into Google Sheets first (File &gt; Import &gt; Upload, replace spreadsheet), Make writes to a live Google Sheet, not a local .xlsx.</t>
@@ -223,19 +223,25 @@
     <t xml:space="preserve">2. Build Scenario 1 (Concept A): trigger module 'LinkedIn Lead Gen Ads' -&gt; 'Watch Leads', connect the LinkedIn Ads account, select the Concept A form specifically.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Action module: 'Google Sheets' -&gt; 'Add a Row', target this spreadsheet's 'Leads' tab. Map Date -&gt; now(), Company/Contact name/Email/Phone -&gt; the matching form fields, and set the 'Concept (A/C)' column to a static value: A.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Build Scenario 2 (Concept C): identical to Scenario 1, but watching the Concept C form, and the 'Concept (A/C)' column set to a static value: C.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Qualified, Sales conversation held, Trial purchased, Repeat purchase, and Revenue are not in LinkedIn's form, leave those blank in both scenarios for manual entry after each lead comes in.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Run each scenario once manually with a test submission before scheduling, confirm the row lands in the right columns with the correct Concept value.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. Turn both scenarios on. From this point, every new form submission on either ad should append a correctly-attributed row automatically.</t>
+    <t xml:space="preserve">3. Action module 1: 'Google Sheets' -&gt; 'Add a Row', target this spreadsheet's 'Leads' tab. Map Date -&gt; now(), Company/Contact name/Email/Phone -&gt; the matching form fields, and set the 'Concept (A/C)' column to a static value: A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Action module 2 (same scenario, runs right after Add a Row): 'Gmail' (or 'Email' module) -&gt; 'Send an Email', to fabien@halostrategic.com. Subject: 'New HVAC lead (Concept A): {{Company}}'. Body: include Company, Contact name, Email, Phone, and a link to this sheet's Leads tab, so Fabien can act within the 15-minute SLA without opening the sheet first.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Build Scenario 2 (Concept C): identical to Scenario 1, but watching the Concept C form, 'Concept (A/C)' set to a static value: C, and the email subject reading 'New HVAC lead (Concept C): {{Company}}'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Qualified, Sales conversation held, Trial purchased, Repeat purchase, and Revenue are not in LinkedIn's form, leave those blank in both scenarios for manual entry after each lead comes in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Run each scenario once manually with a test submission before scheduling, confirm both the sheet row and the email actually arrive correctly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. Turn both scenarios on. From this point, every new form submission on either ad should append a correctly-attributed row AND send Fabien an email, automatically.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email volume note: at a genuinely low lead volume (this is a $300 test), one email per lead is fine. If volume grows later, worth revisiting whether Fabien wants a per-lead email forever or a digest, a decision for that point, not this one.</t>
   </si>
 </sst>
 </file>
@@ -394,7 +400,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -489,6 +495,10 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2693,7 +2703,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="1" style="0" width="30"/>
@@ -2713,7 +2723,7 @@
       <c r="C2" s="22"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="23" t="s">
         <v>63</v>
       </c>
@@ -2721,7 +2731,7 @@
       <c r="C4" s="23"/>
       <c r="D4" s="23"/>
     </row>
-    <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
         <v>64</v>
       </c>
@@ -2729,7 +2739,7 @@
       <c r="C5" s="23"/>
       <c r="D5" s="23"/>
     </row>
-    <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
         <v>65</v>
       </c>
@@ -2737,7 +2747,7 @@
       <c r="C6" s="23"/>
       <c r="D6" s="23"/>
     </row>
-    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
         <v>66</v>
       </c>
@@ -2745,7 +2755,7 @@
       <c r="C7" s="23"/>
       <c r="D7" s="23"/>
     </row>
-    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
         <v>67</v>
       </c>
@@ -2753,7 +2763,7 @@
       <c r="C8" s="23"/>
       <c r="D8" s="23"/>
     </row>
-    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
         <v>68</v>
       </c>
@@ -2761,7 +2771,7 @@
       <c r="C9" s="23"/>
       <c r="D9" s="23"/>
     </row>
-    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="s">
         <v>69</v>
       </c>
@@ -2769,7 +2779,7 @@
       <c r="C10" s="23"/>
       <c r="D10" s="23"/>
     </row>
-    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
         <v>70</v>
       </c>
@@ -2777,8 +2787,24 @@
       <c r="C11" s="23"/>
       <c r="D11" s="23"/>
     </row>
+    <row r="12" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+    </row>
+    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="12">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A4:D4"/>
@@ -2789,6 +2815,8 @@
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>